<commit_message>
feat: ecosistema elevado 10x — 10 MDs + exports + invitaciones verificadas
10 MDs elevados a calidad 10x (sin inflar):
- Ejecutivas ES+EN: criterios aceptacion, 3 escenarios ROI, riesgos, limites
- Detalladas ES+EN: 19 secciones, pricing logic, edge cases, glosario
- KYC: barreras sector, madurez digital, WhatsApp vs email, friccion pago
- Due-diligence: risk scoring, exit scenarios, IP protection, escalacion
- Procurement: switching costs, free tier limits, compliance
- Market-research: timing, TAM validation, SAM sensitivity
- Forecast: sensitivity 3 escenarios, cash flow timing, estacionalidad
- Revenue: break-even sensitivity, capacity ceiling, ambassador funnel, churn

Exports regenerados: 4 DOCX + 2 XLSX + 2 PPTX

Invitaciones verificadas:
- 0 mailto, 0 auto-entrenar, 0 equity viejo
- Masterclass, experiencia, footer homologado en todos
- Countdown correcto (lun 6 abril 7PM)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/propuesta-bootcamp-ejecutivo-quito-2026/outputs/export/comparativa-productos.xlsx
+++ b/propuesta-bootcamp-ejecutivo-quito-2026/outputs/export/comparativa-productos.xlsx
@@ -48,7 +48,7 @@
     <t>Directivos y managers</t>
   </si>
   <si>
-    <t>Agente funcional con contexto real</t>
+    <t>Agente funcional con contexto real (operativo para tareas basicas desde el dia 1)</t>
   </si>
   <si>
     <t>CAO Bootcamp - Edicion Creyentes</t>
@@ -66,7 +66,7 @@
     <t>Directivos C-level, fundadores</t>
   </si>
   <si>
-    <t>1 agente propio (Instalamos a Pristino, agente Open Source desarrollado y mantenido por MetodologIA, obra de Javier Montano. Suyo para siempre, auditable, corre en local)</t>
+    <t>1 agente propio (Instalamos a Pristino, agente Open Source de Javier Montano. En el taller aprende a usarlo en su version basica. Sacarle todo el potencial: auto-estudio o de la mano de nosotros en el Bootcamp. Suyo para siempre, auditable)</t>
   </si>
   <si>
     <t>CAO Bootcamp - Calendario Academico</t>

</xml_diff>